<commit_message>
• Updated cybersecurity requirements per taxonomy and cybersecurity requirement decomposition workbooks (wording change)
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/working_material/cybersecurity requirements decomposition.xlsx
+++ b/distribution/reference_documents/working_material/cybersecurity requirements decomposition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/working_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7E89A0-97E0-DD42-A42E-FA7DA72BA59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25231427-52FA-0A49-A971-7B6B745BEBD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24580" yWindow="3560" windowWidth="27520" windowHeight="27840" xr2:uid="{56895247-3B3D-3147-A316-D5FB82A09ACE}"/>
+    <workbookView xWindow="24580" yWindow="3540" windowWidth="27520" windowHeight="27840" activeTab="3" xr2:uid="{56895247-3B3D-3147-A316-D5FB82A09ACE}"/>
   </bookViews>
   <sheets>
     <sheet name="layer-asset-property sort" sheetId="8" r:id="rId1"/>
@@ -225,9 +225,6 @@
     <t>Configuration data authenticity shall be assured.</t>
   </si>
   <si>
-    <t>Configuration data modification shall be recorded in the audit logs.</t>
-  </si>
-  <si>
     <t>Configuration data modification shall only be made by authorized entities.</t>
   </si>
   <si>
@@ -237,9 +234,6 @@
     <t>Credentials stored in a database shall be encrypted.</t>
   </si>
   <si>
-    <t>Unstructured data security relevant activity shall be recorded in the audit logs.</t>
-  </si>
-  <si>
     <t>Unstructured data access shall be granted based on the principle of least privilege.</t>
   </si>
   <si>
@@ -249,9 +243,6 @@
     <t>Logs shall fully pre-allocate their storage to ensure catastrophic events are recorded.</t>
   </si>
   <si>
-    <t>Security relevant events shall be recorded in the audit logs.</t>
-  </si>
-  <si>
     <t>PII data transmission shall be recorded in the audit log.</t>
   </si>
   <si>
@@ -514,6 +505,15 @@
   </si>
   <si>
     <t>Custom protocols shall use current best practices for authentication and key exchange (NIST SP 800-57, 63B, 131 and 133).</t>
+  </si>
+  <si>
+    <t>Cybersecurity-relevant non-database file activity shall be recorded in the audit log.</t>
+  </si>
+  <si>
+    <t>Configuration data modification shall be recorded in the audit log.</t>
+  </si>
+  <si>
+    <t>Security relevant events shall be recorded in the audit log.</t>
   </si>
 </sst>
 </file>
@@ -956,7 +956,7 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>48</v>
@@ -1057,10 +1057,10 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="7" t="s">
@@ -1093,7 +1093,7 @@
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
         <v>51</v>
@@ -1117,7 +1117,7 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
         <v>49</v>
@@ -1141,7 +1141,7 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
         <v>50</v>
@@ -1165,7 +1165,7 @@
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B7" t="s">
         <v>52</v>
@@ -1189,7 +1189,7 @@
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
         <v>54</v>
@@ -1213,7 +1213,7 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
         <v>55</v>
@@ -1237,7 +1237,7 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B10" t="s">
         <v>53</v>
@@ -1260,7 +1260,7 @@
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
@@ -1285,7 +1285,7 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B12" t="s">
         <v>24</v>
@@ -1309,7 +1309,7 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
         <v>56</v>
@@ -1331,7 +1331,7 @@
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
@@ -1354,7 +1354,7 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B15" t="s">
         <v>35</v>
@@ -1377,7 +1377,7 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
@@ -1401,7 +1401,7 @@
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B17" t="s">
         <v>38</v>
@@ -1425,7 +1425,7 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
@@ -1449,7 +1449,7 @@
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
@@ -1473,10 +1473,10 @@
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="7"/>
@@ -1497,7 +1497,7 @@
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B21" t="s">
         <v>57</v>
@@ -1520,7 +1520,7 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B23" t="s">
         <v>59</v>
@@ -1576,7 +1576,7 @@
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B24" t="s">
         <v>58</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B25" t="s">
         <v>60</v>
@@ -1626,7 +1626,7 @@
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B26" t="s">
         <v>61</v>
@@ -1651,10 +1651,10 @@
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B27" t="s">
-        <v>62</v>
+        <v>157</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="7"/>
@@ -1676,10 +1676,10 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
@@ -1701,10 +1701,10 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>45</v>
@@ -1729,10 +1729,10 @@
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="7"/>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B31" t="s">
         <v>20</v>
@@ -1779,10 +1779,10 @@
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="7"/>
@@ -1804,10 +1804,10 @@
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B33" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="7"/>
@@ -1829,10 +1829,10 @@
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="7"/>
@@ -1854,10 +1854,10 @@
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B35" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="7"/>
@@ -1879,10 +1879,10 @@
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B36" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="7"/>
@@ -1904,7 +1904,7 @@
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B37" t="s">
         <v>31</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B38" t="s">
         <v>32</v>
@@ -1954,7 +1954,7 @@
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B39" t="s">
         <v>11</v>
@@ -1979,7 +1979,7 @@
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B40" t="s">
         <v>33</v>
@@ -2007,10 +2007,10 @@
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B41" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>45</v>
@@ -2032,7 +2032,7 @@
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B42" t="s">
         <v>41</v>
@@ -2057,7 +2057,7 @@
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B43" t="s">
         <v>43</v>
@@ -2082,7 +2082,7 @@
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B44" t="s">
         <v>22</v>
@@ -2107,10 +2107,10 @@
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B45" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C45" s="6"/>
       <c r="D45" s="7"/>
@@ -2132,7 +2132,7 @@
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B46" t="s">
         <v>42</v>
@@ -2157,10 +2157,10 @@
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B47" t="s">
-        <v>70</v>
+        <v>158</v>
       </c>
       <c r="C47" s="6"/>
       <c r="D47" s="7"/>
@@ -2182,7 +2182,7 @@
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B48" t="s">
         <v>30</v>
@@ -2207,10 +2207,10 @@
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B49" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C49" s="6"/>
       <c r="D49" s="7"/>
@@ -2232,7 +2232,7 @@
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B50" t="s">
         <v>28</v>
@@ -2258,10 +2258,10 @@
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B51" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C51" s="6"/>
       <c r="D51" s="7" t="s">
@@ -2284,10 +2284,10 @@
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B52" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>45</v>
@@ -2312,10 +2312,10 @@
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B53" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>45</v>
@@ -2340,10 +2340,10 @@
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B54" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>45</v>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B55" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>45</v>
@@ -2396,10 +2396,10 @@
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B56" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="7" t="s">
@@ -2424,10 +2424,10 @@
     </row>
     <row r="57" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B57" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C57" s="6"/>
       <c r="D57" s="7"/>
@@ -2452,10 +2452,10 @@
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B58" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C58" s="6"/>
       <c r="E58" s="7"/>
@@ -2479,10 +2479,10 @@
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B59" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C59" s="6"/>
       <c r="D59" s="7"/>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B60" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="7"/>
@@ -2529,10 +2529,10 @@
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B61" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>45</v>
@@ -2554,10 +2554,10 @@
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B62" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>45</v>
@@ -2578,7 +2578,7 @@
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B63" t="s">
         <v>36</v>
@@ -2602,7 +2602,7 @@
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
@@ -2626,7 +2626,7 @@
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B65" t="s">
         <v>15</v>
@@ -2673,7 +2673,7 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>48</v>
@@ -2774,10 +2774,10 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="7" t="s">
@@ -2810,7 +2810,7 @@
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
         <v>51</v>
@@ -2834,7 +2834,7 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
         <v>49</v>
@@ -2858,7 +2858,7 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
         <v>50</v>
@@ -2882,7 +2882,7 @@
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B7" t="s">
         <v>52</v>
@@ -2906,7 +2906,7 @@
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
         <v>54</v>
@@ -2930,7 +2930,7 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
         <v>55</v>
@@ -2954,7 +2954,7 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B10" t="s">
         <v>53</v>
@@ -2977,7 +2977,7 @@
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
@@ -3002,7 +3002,7 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B12" t="s">
         <v>24</v>
@@ -3026,7 +3026,7 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
         <v>56</v>
@@ -3048,7 +3048,7 @@
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
@@ -3071,7 +3071,7 @@
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B15" t="s">
         <v>35</v>
@@ -3094,7 +3094,7 @@
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
@@ -3118,7 +3118,7 @@
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B17" t="s">
         <v>38</v>
@@ -3142,7 +3142,7 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
@@ -3166,7 +3166,7 @@
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
@@ -3190,10 +3190,10 @@
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="7"/>
@@ -3214,7 +3214,7 @@
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B21" t="s">
         <v>57</v>
@@ -3237,7 +3237,7 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
@@ -3268,7 +3268,7 @@
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B23" t="s">
         <v>59</v>
@@ -3293,7 +3293,7 @@
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B24" t="s">
         <v>58</v>
@@ -3318,7 +3318,7 @@
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B25" t="s">
         <v>60</v>
@@ -3343,7 +3343,7 @@
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B26" t="s">
         <v>61</v>
@@ -3368,10 +3368,10 @@
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B27" t="s">
-        <v>62</v>
+        <v>157</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="7"/>
@@ -3393,10 +3393,10 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
@@ -3418,10 +3418,10 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>45</v>
@@ -3446,10 +3446,10 @@
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="7"/>
@@ -3471,7 +3471,7 @@
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B31" t="s">
         <v>20</v>
@@ -3496,10 +3496,10 @@
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="7"/>
@@ -3521,10 +3521,10 @@
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B33" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="7"/>
@@ -3546,10 +3546,10 @@
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>45</v>
@@ -3574,10 +3574,10 @@
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B35" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="7"/>
@@ -3599,10 +3599,10 @@
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B36" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="7"/>
@@ -3624,10 +3624,10 @@
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B37" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C37" s="6"/>
       <c r="D37" s="7"/>
@@ -3649,7 +3649,7 @@
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B38" t="s">
         <v>31</v>
@@ -3674,7 +3674,7 @@
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B39" t="s">
         <v>32</v>
@@ -3699,7 +3699,7 @@
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B40" t="s">
         <v>11</v>
@@ -3724,7 +3724,7 @@
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B41" t="s">
         <v>33</v>
@@ -3752,10 +3752,10 @@
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B42" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>45</v>
@@ -3777,7 +3777,7 @@
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B43" t="s">
         <v>41</v>
@@ -3802,7 +3802,7 @@
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B44" t="s">
         <v>43</v>
@@ -3827,7 +3827,7 @@
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B45" t="s">
         <v>22</v>
@@ -3852,10 +3852,10 @@
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B46" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="7"/>
@@ -3877,7 +3877,7 @@
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B47" t="s">
         <v>42</v>
@@ -3902,10 +3902,10 @@
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B48" t="s">
-        <v>70</v>
+        <v>158</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="7"/>
@@ -3927,7 +3927,7 @@
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B49" t="s">
         <v>30</v>
@@ -3952,10 +3952,10 @@
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>45</v>
@@ -3980,10 +3980,10 @@
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B51" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C51" s="6"/>
       <c r="D51" s="7"/>
@@ -4005,10 +4005,10 @@
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B52" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>45</v>
@@ -4033,10 +4033,10 @@
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B53" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>45</v>
@@ -4061,10 +4061,10 @@
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B54" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>45</v>
@@ -4086,10 +4086,10 @@
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B55" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C55" s="6"/>
       <c r="D55" s="7" t="s">
@@ -4114,10 +4114,10 @@
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B56" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="7"/>
@@ -4142,10 +4142,10 @@
     </row>
     <row r="57" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B57" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C57" s="6"/>
       <c r="D57" s="7"/>
@@ -4167,10 +4167,10 @@
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B58" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C58" s="6"/>
       <c r="E58" s="7"/>
@@ -4194,10 +4194,10 @@
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C59" s="6"/>
       <c r="D59" s="7"/>
@@ -4219,7 +4219,7 @@
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B60" t="s">
         <v>28</v>
@@ -4245,10 +4245,10 @@
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B61" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C61" s="6"/>
       <c r="D61" s="7" t="s">
@@ -4271,10 +4271,10 @@
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B62" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>45</v>
@@ -4295,7 +4295,7 @@
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B63" t="s">
         <v>36</v>
@@ -4319,7 +4319,7 @@
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
@@ -4343,7 +4343,7 @@
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B65" t="s">
         <v>15</v>
@@ -4414,30 +4414,30 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>48</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>150</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7" t="s">
@@ -4447,7 +4447,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>51</v>
@@ -4463,7 +4463,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>49</v>
@@ -4479,7 +4479,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>50</v>
@@ -4488,12 +4488,12 @@
         <v>45</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>52</v>
@@ -4509,7 +4509,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>54</v>
@@ -4522,7 +4522,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>55</v>
@@ -4535,7 +4535,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>53</v>
@@ -4548,7 +4548,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>7</v>
@@ -4560,7 +4560,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>24</v>
@@ -4573,7 +4573,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>56</v>
@@ -4585,7 +4585,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>34</v>
@@ -4598,7 +4598,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>35</v>
@@ -4611,7 +4611,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>37</v>
@@ -4624,7 +4624,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>38</v>
@@ -4637,7 +4637,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>25</v>
@@ -4649,7 +4649,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>26</v>
@@ -4662,10 +4662,10 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7" t="s">
@@ -4675,7 +4675,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>57</v>
@@ -4687,7 +4687,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>29</v>
@@ -4700,7 +4700,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>59</v>
@@ -4712,7 +4712,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>58</v>
@@ -4728,7 +4728,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>60</v>
@@ -4740,7 +4740,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>61</v>
@@ -4753,10 +4753,10 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>62</v>
+        <v>157</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="7" t="s">
@@ -4766,24 +4766,24 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>45</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7" t="s">
@@ -4793,10 +4793,10 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>45</v>
@@ -4805,7 +4805,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>20</v>
@@ -4818,10 +4818,10 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>66</v>
+        <v>112</v>
+      </c>
+      <c r="B31" t="s">
+        <v>156</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7" t="s">
@@ -4831,10 +4831,10 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="7" t="s">
@@ -4844,10 +4844,10 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="9" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7" t="s">
@@ -4857,10 +4857,10 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="9" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="7" t="s">
@@ -4870,10 +4870,10 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="7" t="s">
@@ -4883,7 +4883,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="9" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>31</v>
@@ -4896,7 +4896,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>32</v>
@@ -4909,7 +4909,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>11</v>
@@ -4921,7 +4921,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>33</v>
@@ -4934,10 +4934,10 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C40" s="7"/>
       <c r="D40" s="7" t="s">
@@ -4947,7 +4947,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>41</v>
@@ -4960,7 +4960,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B42" s="10" t="s">
         <v>43</v>
@@ -4972,7 +4972,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>22</v>
@@ -4985,10 +4985,10 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C44" s="7"/>
       <c r="D44" s="7" t="s">
@@ -4998,7 +4998,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>42</v>
@@ -5010,10 +5010,10 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="9" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>70</v>
+        <v>158</v>
       </c>
       <c r="C46" s="7"/>
       <c r="D46" s="7" t="s">
@@ -5023,7 +5023,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>30</v>
@@ -5035,10 +5035,10 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="9" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="7" t="s">
@@ -5048,7 +5048,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="9" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>28</v>
@@ -5061,10 +5061,10 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C50" s="7"/>
       <c r="D50" s="7" t="s">
@@ -5074,10 +5074,10 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>45</v>
@@ -5086,10 +5086,10 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="9" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C52" s="7" t="s">
         <v>45</v>
@@ -5098,10 +5098,10 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="7" t="s">
@@ -5111,10 +5111,10 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="9" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C54" s="7" t="s">
         <v>45</v>
@@ -5123,10 +5123,10 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="9" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C55" s="7" t="s">
         <v>45</v>
@@ -5135,10 +5135,10 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C56" s="7"/>
       <c r="D56" s="7" t="s">
@@ -5148,10 +5148,10 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C57" s="7" t="s">
         <v>45</v>
@@ -5160,10 +5160,10 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C58" s="7"/>
       <c r="D58" s="7" t="s">
@@ -5173,10 +5173,10 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C59" s="7"/>
       <c r="D59" s="7" t="s">
@@ -5186,10 +5186,10 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="9" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C60" s="7"/>
       <c r="D60" s="7" t="s">
@@ -5199,10 +5199,10 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="9" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C61" s="7"/>
       <c r="D61" s="7" t="s">
@@ -5212,7 +5212,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="9" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>36</v>
@@ -5228,7 +5228,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>39</v>
@@ -5244,7 +5244,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>15</v>
@@ -5279,27 +5279,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>48</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F1" s="12" t="s">
         <v>150</v>
-      </c>
-      <c r="F1" s="12" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>50</v>
@@ -5308,12 +5308,12 @@
         <v>45</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>7</v>
@@ -5325,7 +5325,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>56</v>
@@ -5337,7 +5337,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>25</v>
@@ -5349,7 +5349,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>57</v>
@@ -5361,7 +5361,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>59</v>
@@ -5373,7 +5373,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>60</v>
@@ -5385,24 +5385,24 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>45</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>45</v>
@@ -5411,7 +5411,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>11</v>
@@ -5423,7 +5423,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>43</v>
@@ -5435,7 +5435,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>42</v>
@@ -5447,7 +5447,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>30</v>
@@ -5459,10 +5459,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>45</v>
@@ -5471,10 +5471,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>45</v>
@@ -5483,10 +5483,10 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>45</v>
@@ -5495,10 +5495,10 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>45</v>
@@ -5507,10 +5507,10 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>45</v>
@@ -5519,10 +5519,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7" t="s">
@@ -5532,7 +5532,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>51</v>
@@ -5548,7 +5548,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>49</v>
@@ -5564,7 +5564,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>52</v>
@@ -5580,7 +5580,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>54</v>
@@ -5593,7 +5593,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>55</v>
@@ -5606,7 +5606,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>53</v>
@@ -5619,7 +5619,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>24</v>
@@ -5632,7 +5632,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>34</v>
@@ -5645,7 +5645,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>35</v>
@@ -5658,7 +5658,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>37</v>
@@ -5671,7 +5671,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>38</v>
@@ -5684,7 +5684,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B32" s="10" t="s">
         <v>26</v>
@@ -5697,10 +5697,10 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="9" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7" t="s">
@@ -5710,7 +5710,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>29</v>
@@ -5723,7 +5723,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>58</v>
@@ -5739,7 +5739,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="9" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>61</v>
@@ -5752,10 +5752,10 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="9" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>62</v>
+        <v>157</v>
       </c>
       <c r="C37" s="7"/>
       <c r="D37" s="7" t="s">
@@ -5765,10 +5765,10 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="9" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C38" s="7"/>
       <c r="D38" s="7" t="s">
@@ -5778,7 +5778,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B39" s="10" t="s">
         <v>20</v>
@@ -5791,10 +5791,10 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>66</v>
+        <v>112</v>
+      </c>
+      <c r="B40" t="s">
+        <v>156</v>
       </c>
       <c r="C40" s="7"/>
       <c r="D40" s="7" t="s">
@@ -5804,10 +5804,10 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C41" s="7"/>
       <c r="D41" s="7" t="s">
@@ -5817,10 +5817,10 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C42" s="7"/>
       <c r="D42" s="7" t="s">
@@ -5830,10 +5830,10 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="9" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C43" s="7"/>
       <c r="D43" s="7" t="s">
@@ -5843,10 +5843,10 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="9" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C44" s="7"/>
       <c r="D44" s="7" t="s">
@@ -5856,7 +5856,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="9" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>31</v>
@@ -5869,7 +5869,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B46" s="10" t="s">
         <v>32</v>
@@ -5882,7 +5882,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>33</v>
@@ -5895,10 +5895,10 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="7" t="s">
@@ -5908,7 +5908,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B49" s="10" t="s">
         <v>41</v>
@@ -5921,7 +5921,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B50" s="10" t="s">
         <v>22</v>
@@ -5934,10 +5934,10 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C51" s="7"/>
       <c r="D51" s="7" t="s">
@@ -5947,10 +5947,10 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="9" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>70</v>
+        <v>158</v>
       </c>
       <c r="C52" s="7"/>
       <c r="D52" s="7" t="s">
@@ -5960,10 +5960,10 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="9" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C53" s="7"/>
       <c r="D53" s="7" t="s">
@@ -5973,7 +5973,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="9" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B54" s="10" t="s">
         <v>28</v>
@@ -5986,10 +5986,10 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="9" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C55" s="7"/>
       <c r="D55" s="7" t="s">
@@ -5999,10 +5999,10 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C56" s="9"/>
       <c r="D56" s="7" t="s">
@@ -6012,10 +6012,10 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C57" s="7"/>
       <c r="D57" s="7" t="s">
@@ -6025,10 +6025,10 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C58" s="7"/>
       <c r="D58" s="7" t="s">
@@ -6038,10 +6038,10 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C59" s="7"/>
       <c r="D59" s="7" t="s">
@@ -6051,10 +6051,10 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="9" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C60" s="7"/>
       <c r="D60" s="7" t="s">
@@ -6064,10 +6064,10 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="9" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C61" s="7"/>
       <c r="D61" s="7" t="s">
@@ -6077,7 +6077,7 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="9" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>36</v>
@@ -6093,7 +6093,7 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>39</v>
@@ -6109,7 +6109,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>15</v>

</xml_diff>